<commit_message>
Demo funcional Back con funcion GPDF agregada kepler-oct-2025
</commit_message>
<xml_diff>
--- a/Demo-oct25/databases/personal_turnos.xlsx
+++ b/Demo-oct25/databases/personal_turnos.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2979</v>
+        <v>156</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1183</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="3">
@@ -494,27 +494,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1236</v>
+        <v>286</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Juan Pérez</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>102</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>María López</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>2387</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Luis Ortega</t>
-        </is>
-      </c>
       <c r="G3" t="n">
-        <v>851</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="4">
@@ -525,7 +525,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -533,19 +533,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3028</v>
+        <v>1082</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1379</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5">
@@ -556,27 +556,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3904</v>
+        <v>724</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>571</v>
+        <v>420</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>78</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6">
@@ -587,27 +587,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1067</v>
+        <v>5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2274</v>
+        <v>1193</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1167</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7">
@@ -618,27 +618,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1416</v>
+        <v>1095</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>255</v>
+        <v>36</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2704</v>
+        <v>590</v>
       </c>
     </row>
     <row r="8">
@@ -649,27 +649,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1053</v>
+        <v>134</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3181</v>
+        <v>561</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>372</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9">
@@ -680,27 +680,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1189</v>
+        <v>1021</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2699</v>
+        <v>108</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>334</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10">
@@ -711,27 +711,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>135</v>
+        <v>103</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3319</v>
+        <v>722</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1192</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>157</v>
+        <v>315</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1912</v>
+        <v>1135</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2135</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -773,27 +773,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3335</v>
+        <v>1072</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>Juan Pérez</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>346</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>María López</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>706</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Luis Ortega</t>
-        </is>
-      </c>
       <c r="G12" t="n">
-        <v>498</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13">
@@ -804,27 +804,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>223</v>
+        <v>1196</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1483</v>
+        <v>595</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>3094</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14">
@@ -835,27 +835,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>182</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3724</v>
+        <v>158</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>881</v>
+        <v>701</v>
       </c>
     </row>
     <row r="15">
@@ -866,27 +866,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2193</v>
+        <v>724</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>788</v>
+        <v>535</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1615</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16">
@@ -897,27 +897,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2788</v>
+        <v>214</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1039</v>
+        <v>815</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>743</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17">
@@ -928,27 +928,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1723</v>
+        <v>678</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>921</v>
+        <v>738</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2109</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18">
@@ -959,27 +959,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>198</v>
+        <v>22</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3393</v>
+        <v>775</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>702</v>
+        <v>707</v>
       </c>
     </row>
     <row r="19">
@@ -990,27 +990,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>873</v>
+        <v>1162</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2853</v>
+        <v>47</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>656</v>
+        <v>741</v>
       </c>
     </row>
     <row r="20">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>100</v>
+        <v>602</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>379</v>
+        <v>757</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3951</v>
+        <v>451</v>
       </c>
     </row>
     <row r="21">
@@ -1052,27 +1052,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>552</v>
+        <v>598</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>Juan Pérez</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>241</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>María López</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>49</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Luis Ortega</t>
-        </is>
-      </c>
       <c r="G21" t="n">
-        <v>4130</v>
+        <v>565</v>
       </c>
     </row>
     <row r="22">
@@ -1083,27 +1083,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2678</v>
+        <v>964</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>692</v>
+        <v>303</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1017</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23">
@@ -1114,27 +1114,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1096</v>
+        <v>308</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>51</v>
+        <v>735</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>3112</v>
+        <v>730</v>
       </c>
     </row>
     <row r="24">
@@ -1145,27 +1145,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3823</v>
+        <v>611</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>530</v>
+        <v>219</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>27</v>
+        <v>563</v>
       </c>
     </row>
     <row r="25">
@@ -1176,27 +1176,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2968</v>
+        <v>93</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>761</v>
+        <v>692</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>849</v>
+        <v>366</v>
       </c>
     </row>
     <row r="26">
@@ -1207,27 +1207,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1027</v>
+        <v>698</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>853</v>
+        <v>146</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2568</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27">
@@ -1238,27 +1238,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2243</v>
+        <v>52</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>786</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28">
@@ -1269,27 +1269,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1928</v>
+        <v>235</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1350</v>
+        <v>91</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1017</v>
+        <v>921</v>
       </c>
     </row>
     <row r="29">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>164</v>
+        <v>476</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1998</v>
+        <v>612</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>2060</v>
+        <v>878</v>
       </c>
     </row>
     <row r="30">
@@ -1331,27 +1331,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1227</v>
+        <v>93</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>Juan Pérez</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>579</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>María López</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>2144</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Luis Ortega</t>
-        </is>
-      </c>
       <c r="G30" t="n">
-        <v>1316</v>
+        <v>484</v>
       </c>
     </row>
     <row r="31">
@@ -1362,27 +1362,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1367</v>
+        <v>77</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>María López</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1891</v>
+        <v>972</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1426</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -1444,27 +1444,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1347</v>
+        <v>355</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>113</v>
+        <v>637</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2740</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3">
@@ -1475,27 +1475,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>935</v>
+        <v>468</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2430</v>
+        <v>148</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1109</v>
+        <v>814</v>
       </c>
     </row>
     <row r="4">
@@ -1506,27 +1506,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2786</v>
+        <v>115</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1013</v>
+        <v>252</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>735</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="5">
@@ -1537,27 +1537,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1360</v>
+        <v>555</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2343</v>
+        <v>184</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>850</v>
+        <v>624</v>
       </c>
     </row>
     <row r="6">
@@ -1568,27 +1568,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3724</v>
+        <v>982</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>53</v>
+        <v>131</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>730</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7">
@@ -1599,27 +1599,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3143</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>727</v>
+        <v>937</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>504</v>
+        <v>784</v>
       </c>
     </row>
     <row r="8">
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1285</v>
+        <v>129</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1311</v>
+        <v>549</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2011</v>
+        <v>476</v>
       </c>
     </row>
     <row r="9">
@@ -1661,27 +1661,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>939</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>446</v>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="n">
+        <v>250</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>José Rivas</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>939</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G9" t="n">
-        <v>2838</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10">
@@ -1692,27 +1692,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>María López</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>163</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>219</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>3010</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>José Rivas</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1230</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G10" t="n">
-        <v>406</v>
+        <v>726</v>
       </c>
     </row>
     <row r="11">
@@ -1723,27 +1723,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1737</v>
+        <v>880</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2053</v>
+        <v>114</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>415</v>
+        <v>498</v>
       </c>
     </row>
     <row r="12">
@@ -1754,27 +1754,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1119</v>
+        <v>178</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1802</v>
+        <v>749</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1618</v>
+        <v>783</v>
       </c>
     </row>
     <row r="13">
@@ -1785,27 +1785,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2489</v>
+        <v>48</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1781</v>
+        <v>1831</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>531</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14">
@@ -1816,27 +1816,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>50</v>
+        <v>907</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2922</v>
+        <v>127</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1724</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1847,27 +1847,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>427</v>
+        <v>257</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3067</v>
+        <v>611</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1102</v>
+        <v>693</v>
       </c>
     </row>
     <row r="16">
@@ -1878,27 +1878,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2113</v>
+        <v>441</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2178</v>
+        <v>346</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>278</v>
+        <v>469</v>
       </c>
     </row>
     <row r="17">
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>250</v>
+        <v>1117</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2402</v>
+        <v>104</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2101</v>
+        <v>574</v>
       </c>
     </row>
     <row r="18">
@@ -1940,27 +1940,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>164</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>219</v>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="n">
+        <v>963</v>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>José Rivas</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>2680</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G18" t="n">
-        <v>1394</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19">
@@ -1971,27 +1971,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>María López</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1268</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>157</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>81</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>José Rivas</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1815</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G19" t="n">
-        <v>2486</v>
+        <v>524</v>
       </c>
     </row>
     <row r="20">
@@ -2002,27 +2002,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3536</v>
+        <v>1171</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>36</v>
+        <v>119</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>858</v>
+        <v>519</v>
       </c>
     </row>
     <row r="21">
@@ -2033,27 +2033,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>682</v>
+        <v>472</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1057</v>
+        <v>775</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2992</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22">
@@ -2064,27 +2064,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1023</v>
+        <v>104</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1593</v>
+        <v>519</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1771</v>
+        <v>694</v>
       </c>
     </row>
     <row r="23">
@@ -2095,27 +2095,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2952</v>
+        <v>226</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>899</v>
+        <v>53</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>407</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="24">
@@ -2126,27 +2126,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>766</v>
+        <v>231</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>3374</v>
+        <v>332</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>240</v>
+        <v>830</v>
       </c>
     </row>
     <row r="25">
@@ -2157,27 +2157,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1776</v>
+        <v>482</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>655</v>
+        <v>569</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Lucía Díaz</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2147</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2019</v>
+        <v>352</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2155</v>
+        <v>537</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>274</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27">
@@ -2219,27 +2219,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>68</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C27" t="n">
-        <v>2952</v>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="n">
+        <v>1438</v>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>José Rivas</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>1110</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G27" t="n">
-        <v>534</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28">
@@ -2250,27 +2250,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>María López</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>40</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Luis Ortega</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>754</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>Ana Torres</t>
         </is>
       </c>
-      <c r="C28" t="n">
-        <v>2239</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>José Rivas</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1194</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Raúl Gómez</t>
-        </is>
-      </c>
       <c r="G28" t="n">
-        <v>863</v>
+        <v>454</v>
       </c>
     </row>
     <row r="29">
@@ -2281,27 +2281,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2703</v>
+        <v>507</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>633</v>
+        <v>1330</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>887</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30">
@@ -2312,27 +2312,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1933</v>
+        <v>111</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>992</v>
+        <v>409</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1762</v>
+        <v>637</v>
       </c>
     </row>
     <row r="31">
@@ -2343,27 +2343,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1086</v>
+        <v>568</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>José Rivas</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1731</v>
+        <v>151</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Raúl Gómez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1868</v>
+        <v>640</v>
       </c>
     </row>
   </sheetData>
@@ -2425,27 +2425,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1716</v>
+        <v>395</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1352</v>
+        <v>570</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1133</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3">
@@ -2456,27 +2456,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>847</v>
+        <v>648</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1597</v>
+        <v>509</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2030</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4">
@@ -2487,27 +2487,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>278</v>
+        <v>571</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2415</v>
+        <v>737</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1842</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1181</v>
+        <v>306</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2780</v>
+        <v>558</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2538,7 +2538,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>592</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6">
@@ -2549,27 +2549,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1485</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>581</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="n">
+        <v>55</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Carlos Vega</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>66</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G6" t="n">
-        <v>3861</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -2580,27 +2580,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>José Rivas</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>879</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>254</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>2754</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Carlos Vega</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>319</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G7" t="n">
-        <v>1302</v>
+        <v>589</v>
       </c>
     </row>
     <row r="8">
@@ -2611,27 +2611,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>716</v>
+        <v>523</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1660</v>
+        <v>490</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2231</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
@@ -2642,27 +2642,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>209</v>
+        <v>441</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3296</v>
+        <v>401</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>718</v>
+        <v>570</v>
       </c>
     </row>
     <row r="10">
@@ -2673,27 +2673,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>525</v>
+        <v>63</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1447</v>
+        <v>196</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2674</v>
+        <v>850</v>
       </c>
     </row>
     <row r="11">
@@ -2704,27 +2704,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3576</v>
+        <v>276</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>66</v>
+        <v>981</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>563</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12">
@@ -2735,27 +2735,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>724</v>
+        <v>286</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2623</v>
+        <v>689</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1192</v>
+        <v>735</v>
       </c>
     </row>
     <row r="13">
@@ -2766,27 +2766,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2787</v>
+        <v>1335</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1316</v>
+        <v>174</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>697</v>
+        <v>462</v>
       </c>
     </row>
     <row r="14">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1373</v>
+        <v>375</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1985</v>
+        <v>647</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1337</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -2828,27 +2828,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1318</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>2877</v>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="n">
+        <v>160</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>Carlos Vega</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>156</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G15" t="n">
-        <v>1564</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16">
@@ -2859,27 +2859,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>José Rivas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>410</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>262</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>1368</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Carlos Vega</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>2385</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G16" t="n">
-        <v>816</v>
+        <v>583</v>
       </c>
     </row>
     <row r="17">
@@ -2890,27 +2890,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>223</v>
+        <v>351</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>123</v>
+        <v>703</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>4407</v>
+        <v>742</v>
       </c>
     </row>
     <row r="18">
@@ -2921,27 +2921,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>589</v>
+        <v>1352</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>952</v>
+        <v>26</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2752</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19">
@@ -2952,27 +2952,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>127</v>
+        <v>347</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3077</v>
+        <v>513</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1179</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="20">
@@ -2983,27 +2983,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>360</v>
+        <v>298</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1060</v>
+        <v>321</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3010</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="21">
@@ -3014,27 +3014,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>579</v>
+        <v>1259</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3734</v>
+        <v>34</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>418</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22">
@@ -3045,27 +3045,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1664</v>
+        <v>792</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>600</v>
+        <v>316</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2124</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23">
@@ -3080,7 +3080,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3794</v>
+        <v>236</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>295</v>
+        <v>263</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -3096,7 +3096,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>169</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="24">
@@ -3107,27 +3107,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>93</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>2670</v>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="n">
+        <v>787</v>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Carlos Vega</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>255</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G24" t="n">
-        <v>1455</v>
+        <v>513</v>
       </c>
     </row>
     <row r="25">
@@ -3138,27 +3138,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>José Rivas</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>340</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Raúl Gómez</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>526</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Lucía Díaz</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>1619</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Carlos Vega</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>1052</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Rosa Ramírez</t>
-        </is>
-      </c>
       <c r="G25" t="n">
-        <v>1907</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26">
@@ -3169,27 +3169,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2353</v>
+        <v>919</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>847</v>
+        <v>82</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Raúl Gómez</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>1247</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -3200,27 +3200,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3004</v>
+        <v>1366</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1007</v>
+        <v>298</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>José Rivas</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>585</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28">
@@ -3231,27 +3231,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1173</v>
+        <v>230</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1480</v>
+        <v>23</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Ana Torres</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1642</v>
+        <v>994</v>
       </c>
     </row>
     <row r="29">
@@ -3262,27 +3262,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>261</v>
+        <v>37</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2370</v>
+        <v>1157</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1592</v>
+        <v>772</v>
       </c>
     </row>
     <row r="30">
@@ -3293,27 +3293,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>587</v>
+        <v>767</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3826</v>
+        <v>273</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>María López</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>274</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31">
@@ -3324,27 +3324,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lucía Díaz</t>
+          <t>Carlos Vega</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1036</v>
+        <v>698</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Carlos Vega</t>
+          <t>Rosa Ramírez</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>972</v>
+        <v>318</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Rosa Ramírez</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>2676</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>